<commit_message>
Auto update from NIGHT script
</commit_message>
<xml_diff>
--- a/data/Supplement.xlsx
+++ b/data/Supplement.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ortholitevietnam.sharepoint.com/sites/production9/Shared Documents/PRODUCTION/TRUONG OFFICE/WEEKLY REPORT/WE ARE BETTER/vercel-dashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_DB61266FACF10F39B66C813355FDBEEA58404ACA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0DFC8C62-3FAC-4ADF-80CD-EB6463F7C8F7}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_D49781AC3DCA5FE5FFCC362AE99D049711BC364F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4242842C-5A0F-45C4-936D-A21259A96D63}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,9 +17,6 @@
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -35,11 +32,15 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -73,7 +74,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -96,44 +97,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -163,12 +164,12 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -207,155 +208,227 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
+                <a:tint val="100000"/>
                 <a:shade val="100000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="3" ht="15.75" x14ac:dyDescent="0.25"/>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ABA881C598A1DC4096D4B66B961FB704" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="00a272c57818f5a2598402ed9b64a3e4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b65cb79d-c821-4d3d-aab2-5ef15e9cc85e" xmlns:ns3="71b44b8b-5734-40bc-bcd6-983774da7c1c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cb7fe868ff501d2f097cc8d8c004abe7" ns2:_="" ns3:_="">
     <xsd:import namespace="b65cb79d-c821-4d3d-aab2-5ef15e9cc85e"/>
@@ -616,29 +689,28 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="b65cb79d-c821-4d3d-aab2-5ef15e9cc85e">
       <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="71b44b8b-5734-40bc-bcd6-983774da7c1c" xsi:nil="true"/>
     <_Flow_SignoffStatus xmlns="b65cb79d-c821-4d3d-aab2-5ef15e9cc85e" xsi:nil="true"/>
-    <TaxCatchAll xmlns="71b44b8b-5734-40bc-bcd6-983774da7c1c" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{72BDBC8C-268D-46DC-950E-B83A27DCD0DB}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CCDFE4C4-5B96-4C00-9C27-BAA4B256509C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E0E60A91-C509-4872-9DF7-38C7066FAABE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
@@ -656,8 +728,8 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{65580776-39A1-4F81-92E4-469352F66D91}">
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82A14EE1-59CC-47A3-BB1A-D631CBDCDEB8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
@@ -665,12 +737,4 @@
     <ds:schemaRef ds:uri="71b44b8b-5734-40bc-bcd6-983774da7c1c"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8384541B-BAD0-4494-AED6-1A7611440316}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Auto NIGHT update at 2025-08-25 23:36:11
</commit_message>
<xml_diff>
--- a/data/Supplement.xlsx
+++ b/data/Supplement.xlsx
@@ -1,40 +1,201 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29212"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_3149407D34AAD0E3C6A7FEF72B9A1564395F9124" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FC6CB8D2-9852-434A-BFBC-8172FFCD6E6D}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Supplement" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="191028" refMode="R1C1" iterateCount="0" calcOnSave="0" concurrentCalc="0"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="53">
+  <si>
+    <t>RPRO</t>
+  </si>
+  <si>
+    <t>Giới tính</t>
+  </si>
+  <si>
+    <t>Mã khuôn</t>
+  </si>
+  <si>
+    <t>Mã dao</t>
+  </si>
+  <si>
+    <t>Vải</t>
+  </si>
+  <si>
+    <t>BOM</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
+  </si>
+  <si>
+    <t>created_at</t>
+  </si>
+  <si>
+    <t>RPRO-250626-0096</t>
+  </si>
+  <si>
+    <t>Men's</t>
+  </si>
+  <si>
+    <t>DIE-CUT</t>
+  </si>
+  <si>
+    <t>JV1-0695-3(arch skive)</t>
+  </si>
+  <si>
+    <t>145-17-00 LJ-B1-1-VEPM5 44" 180G</t>
+  </si>
+  <si>
+    <t>DC-010097</t>
+  </si>
+  <si>
+    <t>23/07/2025 13:25:54</t>
+  </si>
+  <si>
+    <t>RPRO-250526-0514</t>
+  </si>
+  <si>
+    <t>Women's</t>
+  </si>
+  <si>
+    <t>OE-0198</t>
+  </si>
+  <si>
+    <t>QD-39 (M-0502)</t>
+  </si>
+  <si>
+    <t>71R EPM MERRY MESH(LJB-730) 44" 220G</t>
+  </si>
+  <si>
+    <t>OE-007434</t>
+  </si>
+  <si>
+    <t>23/07/2025 14:24:36</t>
+  </si>
+  <si>
+    <t>RPRO-250610-0389</t>
+  </si>
+  <si>
+    <t>OV-0256</t>
+  </si>
+  <si>
+    <t>21-005-M-Low (M-0235)</t>
+  </si>
+  <si>
+    <t>19-1624TCX YH-S817A EPM5 (100% REC.PES) 44" 220G</t>
+  </si>
+  <si>
+    <t>OV-008378</t>
+  </si>
+  <si>
+    <t>23/07/2025 16:19:54</t>
+  </si>
+  <si>
+    <t>RPRO-250606-0428</t>
+  </si>
+  <si>
+    <t>ON-112 (M-0236)</t>
+  </si>
+  <si>
+    <t>19-3911TCX YH-S817A EPM5 (100% REC.PES) 44" 220G</t>
+  </si>
+  <si>
+    <t>OV-008350</t>
+  </si>
+  <si>
+    <t>23/07/2025 22:26:03</t>
+  </si>
+  <si>
+    <t>RPRO-250627-0145</t>
+  </si>
+  <si>
+    <t>QA-7H (D-0256) (skive arch)</t>
+  </si>
+  <si>
+    <t>10A (PP)LINING KNIT MATTE MICRO (HOOD) REC 44" 250G</t>
+  </si>
+  <si>
+    <t>DC-011263</t>
+  </si>
+  <si>
+    <t>23/07/2025 22:58:44</t>
+  </si>
+  <si>
+    <t>RPRO-250606-0433</t>
+  </si>
+  <si>
+    <t>11-4202TPG YH-S817A EPM5 (100% REC.PES) 44" 220G</t>
+  </si>
+  <si>
+    <t>OV-007210</t>
+  </si>
+  <si>
+    <t>23/07/2025 23:39:58</t>
+  </si>
+  <si>
+    <t>RPRO-250610-0266</t>
+  </si>
+  <si>
+    <t>21-005-W-Low (M-0234)</t>
+  </si>
+  <si>
+    <t>18-4006TPG YH-S817A EPM5 (100% REC.PES) 44" 220G</t>
+  </si>
+  <si>
+    <t>OV-007160</t>
+  </si>
+  <si>
+    <t>24/07/2025 08:23:48</t>
+  </si>
+  <si>
+    <t>RPRO-250610-0514</t>
+  </si>
+  <si>
+    <t>OV-0377</t>
+  </si>
+  <si>
+    <t>ON-8-W-2 (M-0418)</t>
+  </si>
+  <si>
+    <t>11-4202TCX YH-S960 EPM5 (100% Recycled PET) 44'' 198G</t>
+  </si>
+  <si>
+    <t>OV-008950</t>
+  </si>
+  <si>
+    <t>24/07/2025 09:07:49</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1">
     <font>
       <sz val="12"/>
@@ -65,13 +226,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,33 +565,34 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CB10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:CB9"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>RPRO</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Giới tính</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Mã khuôn</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Mã dao</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Vải</v>
-      </c>
-      <c r="F1" t="str">
-        <v>BOM</v>
-      </c>
-      <c r="G1" t="str">
-        <v>TOTAL</v>
-      </c>
-      <c r="H1" t="str">
-        <v>created_at</v>
+    <row r="1" spans="1:80">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
       </c>
       <c r="I1">
         <v>1</v>
@@ -681,30 +851,30 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>RPRO-250626-0096</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Men's</v>
-      </c>
-      <c r="C2" t="str">
-        <v>DIE-CUT</v>
-      </c>
-      <c r="D2" t="str">
-        <v>JV1-0695-3(arch skive)</v>
-      </c>
-      <c r="E2" t="str">
-        <v>145-17-00 LJ-B1-1-VEPM5 44" 180G</v>
-      </c>
-      <c r="F2" t="str">
-        <v>DC-010097</v>
+    <row r="2" spans="1:80">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>13</v>
       </c>
       <c r="G2">
         <v>11</v>
       </c>
-      <c r="H2" t="str">
-        <v>23/07/2025 13:25:54</v>
+      <c r="H2" t="s">
+        <v>14</v>
       </c>
       <c r="I2">
         <v>0</v>
@@ -923,30 +1093,30 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>RPRO-250526-0514</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Women's</v>
-      </c>
-      <c r="C3" t="str">
-        <v>OE-0198</v>
-      </c>
-      <c r="D3" t="str">
-        <v>QD-39 (M-0502)</v>
-      </c>
-      <c r="E3" t="str">
-        <v>71R EPM MERRY MESH(LJB-730) 44" 220G</v>
-      </c>
-      <c r="F3" t="str">
-        <v>OE-007434</v>
+    <row r="3" spans="1:80">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>20</v>
       </c>
       <c r="G3">
         <v>1</v>
       </c>
-      <c r="H3" t="str">
-        <v>23/07/2025 14:24:36</v>
+      <c r="H3" t="s">
+        <v>21</v>
       </c>
       <c r="I3">
         <v>0</v>
@@ -1165,30 +1335,30 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>RPRO-250610-0389</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Men's</v>
-      </c>
-      <c r="C4" t="str">
-        <v>OV-0256</v>
-      </c>
-      <c r="D4" t="str">
-        <v>21-005-M-Low (M-0235)</v>
-      </c>
-      <c r="E4" t="str">
-        <v>19-1624TCX YH-S817A EPM5 (100% REC.PES) 44" 220G</v>
-      </c>
-      <c r="F4" t="str">
-        <v>OV-008378</v>
+    <row r="4" spans="1:80">
+      <c r="A4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" t="s">
+        <v>26</v>
       </c>
       <c r="G4">
         <v>26</v>
       </c>
-      <c r="H4" t="str">
-        <v>23/07/2025 16:19:54</v>
+      <c r="H4" t="s">
+        <v>27</v>
       </c>
       <c r="I4">
         <v>0</v>
@@ -1407,30 +1577,30 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>RPRO-250606-0428</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Men's</v>
-      </c>
-      <c r="C5" t="str">
-        <v>OV-0256</v>
-      </c>
-      <c r="D5" t="str">
-        <v>ON-112 (M-0236)</v>
-      </c>
-      <c r="E5" t="str">
-        <v>19-3911TCX YH-S817A EPM5 (100% REC.PES) 44" 220G</v>
-      </c>
-      <c r="F5" t="str">
-        <v>OV-008350</v>
+    <row r="5" spans="1:80">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5" t="s">
+        <v>31</v>
       </c>
       <c r="G5">
         <v>4</v>
       </c>
-      <c r="H5" t="str">
-        <v>23/07/2025 22:26:03</v>
+      <c r="H5" t="s">
+        <v>32</v>
       </c>
       <c r="I5">
         <v>0</v>
@@ -1649,30 +1819,30 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>RPRO-250627-0145</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Women's</v>
-      </c>
-      <c r="C6" t="str">
-        <v>DIE-CUT</v>
-      </c>
-      <c r="D6" t="str">
-        <v>QA-7H (D-0256) (skive arch)</v>
-      </c>
-      <c r="E6" t="str">
-        <v>10A (PP)LINING KNIT MATTE MICRO (HOOD) REC 44" 250G</v>
-      </c>
-      <c r="F6" t="str">
-        <v>DC-011263</v>
+    <row r="6" spans="1:80">
+      <c r="A6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" t="s">
+        <v>35</v>
+      </c>
+      <c r="F6" t="s">
+        <v>36</v>
       </c>
       <c r="G6">
         <v>2</v>
       </c>
-      <c r="H6" t="str">
-        <v>23/07/2025 22:58:44</v>
+      <c r="H6" t="s">
+        <v>37</v>
       </c>
       <c r="I6">
         <v>0</v>
@@ -1891,30 +2061,30 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>RPRO-250606-0433</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Women's</v>
-      </c>
-      <c r="C7" t="str">
-        <v>OV-0256</v>
-      </c>
-      <c r="D7" t="str">
-        <v>ON-112 (M-0236)</v>
-      </c>
-      <c r="E7" t="str">
-        <v>11-4202TPG YH-S817A EPM5 (100% REC.PES) 44" 220G</v>
-      </c>
-      <c r="F7" t="str">
-        <v>OV-007210</v>
+    <row r="7" spans="1:80">
+      <c r="A7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" t="s">
+        <v>29</v>
+      </c>
+      <c r="E7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F7" t="s">
+        <v>40</v>
       </c>
       <c r="G7">
         <v>0</v>
       </c>
-      <c r="H7" t="str">
-        <v>23/07/2025 23:39:58</v>
+      <c r="H7" t="s">
+        <v>41</v>
       </c>
       <c r="I7">
         <v>0</v>
@@ -2133,30 +2303,30 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>RPRO-250610-0266</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Women's</v>
-      </c>
-      <c r="C8" t="str">
-        <v>OV-0256</v>
-      </c>
-      <c r="D8" t="str">
-        <v>21-005-W-Low (M-0234)</v>
-      </c>
-      <c r="E8" t="str">
-        <v>18-4006TPG YH-S817A EPM5 (100% REC.PES) 44" 220G</v>
-      </c>
-      <c r="F8" t="str">
-        <v>OV-007160</v>
+    <row r="8" spans="1:80">
+      <c r="A8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" t="s">
+        <v>43</v>
+      </c>
+      <c r="E8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F8" t="s">
+        <v>45</v>
       </c>
       <c r="G8">
         <v>210</v>
       </c>
-      <c r="H8" t="str">
-        <v>24/07/2025 08:23:48</v>
+      <c r="H8" t="s">
+        <v>46</v>
       </c>
       <c r="I8">
         <v>0</v>
@@ -2375,30 +2545,30 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>RPRO-250610-0514</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Women's</v>
-      </c>
-      <c r="C9" t="str">
-        <v>OV-0377</v>
-      </c>
-      <c r="D9" t="str">
-        <v>ON-8-W-2 (M-0418)</v>
-      </c>
-      <c r="E9" t="str">
-        <v>11-4202TCX YH-S960 EPM5 (100% Recycled PET) 44'' 198G</v>
-      </c>
-      <c r="F9" t="str">
-        <v>OV-008950</v>
+    <row r="9" spans="1:80">
+      <c r="A9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" t="s">
+        <v>48</v>
+      </c>
+      <c r="D9" t="s">
+        <v>49</v>
+      </c>
+      <c r="E9" t="s">
+        <v>50</v>
+      </c>
+      <c r="F9" t="s">
+        <v>51</v>
       </c>
       <c r="G9">
         <v>23</v>
       </c>
-      <c r="H9" t="str">
-        <v>24/07/2025 09:07:49</v>
+      <c r="H9" t="s">
+        <v>52</v>
       </c>
       <c r="I9">
         <v>0</v>
@@ -2620,14 +2790,23 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:CB10"/>
+    <ignoredError sqref="A1:CB10" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ABA881C598A1DC4096D4B66B961FB704" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="00a272c57818f5a2598402ed9b64a3e4">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b65cb79d-c821-4d3d-aab2-5ef15e9cc85e" xmlns:ns3="71b44b8b-5734-40bc-bcd6-983774da7c1c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cb7fe868ff501d2f097cc8d8c004abe7" ns2:_="" ns3:_="">
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ABA881C598A1DC4096D4B66B961FB704" ma:contentTypeVersion="21" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="63da96a68aea1e0a95bb00dc613529db">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b65cb79d-c821-4d3d-aab2-5ef15e9cc85e" xmlns:ns3="71b44b8b-5734-40bc-bcd6-983774da7c1c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="bc38e99d4a2ab748d495d1563ca7dbf9" ns2:_="" ns3:_="">
     <xsd:import namespace="b65cb79d-c821-4d3d-aab2-5ef15e9cc85e"/>
     <xsd:import namespace="71b44b8b-5734-40bc-bcd6-983774da7c1c"/>
     <xsd:element name="properties">
@@ -2654,6 +2833,7 @@
                 <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
                 <xsd:element ref="ns2:_Flow_SignoffStatus" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -2741,6 +2921,11 @@
       </xsd:simpleType>
     </xsd:element>
     <xsd:element name="MediaServiceSearchProperties" ma:index="26" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="27" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
@@ -2886,15 +3071,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2908,11 +3084,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31919BC8-9379-4D37-B41C-E8135171CD65}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{78549BE0-398A-4CF5-810D-3FEC6A11E863}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{78549BE0-398A-4CF5-810D-3FEC6A11E863}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E9D90A7-B992-4CC5-892A-22FF1C23215E}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>